<commit_message>
Auto update Pengadaan 2026-09-18 08:08:18
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-18).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-18).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1301651478</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>178</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2214983750</v>
+        <v>2224487903</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>11</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>263794708</v>
+        <v>289324708</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>11</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>94995000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>79574469</v>
+        <v>23225929</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>18</v>
@@ -3363,22 +3371,22 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3959</v>
+        <v>3932</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32548022052</v>
+        <v>32583056205</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>423</v>
+        <v>396</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6337114407</v>
+        <v>6372148560</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>423</v>
+        <v>396</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>8937298499.6</v>
+        <v>5899017183.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3536</v>
@@ -5588,28 +5596,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>595373450</v>
+      </c>
+      <c r="E44" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D44" s="9" t="n">
-        <v>379426400</v>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="F44" s="9" t="n">
-        <v>201970600</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>142419460</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>142419460</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -7540,28 +7548,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>95905605114</v>
+        <v>96121552164</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>63623989343</v>
+        <v>63839936393</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>62077269544.41</v>
+        <v>62133618084.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>29411140755</v>
+        <v>29467489295</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>11</v>
@@ -8375,28 +8383,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26485477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26485477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26035273641</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25036544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25036544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24238773641</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24238773641</v>
+        <v>26035273641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8594,13 +8602,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8819,34 +8827,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1613354372</v>
+        <v>2704201180</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12021,34 +12029,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>209</v>
+        <v>233</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>133845825146</v>
+        <v>178281187883</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>96387818241</v>
+        <v>140823180978</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>66292136025.01</v>
+        <v>69274068801.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>61843702225</v>
+        <v>64825635001</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2662960246</v>
+        <v>3753807054</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>79</v>

</xml_diff>